<commit_message>
feat: setup backend base repo and add team conventions (git, backend, frontend)
</commit_message>
<xml_diff>
--- a/docs/scrum/DriveShare_TienDo.xlsx
+++ b/docs/scrum/DriveShare_TienDo.xlsx
@@ -938,7 +938,6 @@
       </c>
       <c r="H9" s="19" t="n"/>
     </row>
-    <row r="10"/>
     <row r="11" ht="27.75" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -1111,7 +1110,6 @@
       </c>
       <c r="H15" s="19" t="n"/>
     </row>
-    <row r="16"/>
     <row r="17" ht="27.75" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
@@ -1432,7 +1430,6 @@
       </c>
       <c r="H25" s="19" t="n"/>
     </row>
-    <row r="26"/>
     <row r="27" ht="27.75" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
         <is>
@@ -1604,7 +1601,6 @@
       </c>
       <c r="H31" s="19" t="n"/>
     </row>
-    <row r="32"/>
     <row r="33" ht="27.75" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
         <is>
@@ -1924,7 +1920,6 @@
       </c>
       <c r="H41" s="19" t="n"/>
     </row>
-    <row r="42"/>
     <row r="43" ht="27.75" customHeight="1">
       <c r="A43" s="4" t="inlineStr">
         <is>
@@ -2096,7 +2091,6 @@
       </c>
       <c r="H47" s="19" t="n"/>
     </row>
-    <row r="48"/>
     <row r="49" ht="27.75" customHeight="1">
       <c r="A49" s="4" t="inlineStr">
         <is>
@@ -2415,7 +2409,6 @@
       </c>
       <c r="H57" s="19" t="n"/>
     </row>
-    <row r="58"/>
     <row r="59" ht="27.75" customHeight="1">
       <c r="A59" s="4" t="inlineStr">
         <is>
@@ -2586,7 +2579,6 @@
       </c>
       <c r="H63" s="19" t="n"/>
     </row>
-    <row r="64"/>
     <row r="65" ht="27.75" customHeight="1">
       <c r="A65" s="4" t="inlineStr">
         <is>
@@ -2756,7 +2748,6 @@
       </c>
       <c r="H69" s="19" t="n"/>
     </row>
-    <row r="70"/>
     <row r="71" ht="27.75" customHeight="1">
       <c r="A71" s="4" t="inlineStr">
         <is>
@@ -2929,7 +2920,6 @@
       </c>
       <c r="H75" s="19" t="n"/>
     </row>
-    <row r="76"/>
     <row r="77" ht="27.75" customHeight="1">
       <c r="A77" s="4" t="inlineStr">
         <is>
@@ -3102,7 +3092,6 @@
       </c>
       <c r="H81" s="19" t="n"/>
     </row>
-    <row r="82"/>
     <row r="83" ht="27.75" customHeight="1">
       <c r="A83" s="4" t="inlineStr">
         <is>
@@ -3739,7 +3728,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="9.285714285714286" customWidth="1" min="1" max="1"/>
@@ -3801,21 +3790,25 @@
       </c>
       <c r="B4" s="26" t="inlineStr">
         <is>
-          <t>Vĩ</t>
-        </is>
-      </c>
-      <c r="C4" s="28" t="n"/>
+          <t>Bảo</t>
+        </is>
+      </c>
+      <c r="C4" s="28" t="inlineStr"/>
       <c r="D4" s="25" t="inlineStr">
         <is>
-          <t>Project Lead / Fullstack</t>
+          <t>Project Lead / Database</t>
         </is>
       </c>
       <c r="E4" s="26" t="inlineStr">
         <is>
-          <t>Sprint 0 (Lead &amp; DB), Admin UI (US-14), Review &amp; Merge PR</t>
-        </is>
-      </c>
-      <c r="F4" s="26" t="n"/>
+          <t>Quản lý dự án, Thiết kế &amp; Tối ưu CSDL v2, Review &amp; Merge PR, CI/CD, Điều phối chung</t>
+        </is>
+      </c>
+      <c r="F4" s="26" t="inlineStr">
+        <is>
+          <t>Lead &amp; Data Architect</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="24.75" customHeight="1">
       <c r="A5" s="28" t="n">
@@ -3823,21 +3816,25 @@
       </c>
       <c r="B5" s="26" t="inlineStr">
         <is>
-          <t>Phát</t>
-        </is>
-      </c>
-      <c r="C5" s="28" t="n"/>
+          <t>Lộc Khiêm</t>
+        </is>
+      </c>
+      <c r="C5" s="28" t="inlineStr"/>
       <c r="D5" s="25" t="inlineStr">
         <is>
-          <t>Backend Developer</t>
+          <t>Backend Developer (Core Transaction Engine)</t>
         </is>
       </c>
       <c r="E5" s="26" t="inlineStr">
         <is>
-          <t>Sprint 0 (Luồng 1), BE Core: US-01, US-03, US-04, US-05, US-06</t>
-        </is>
-      </c>
-      <c r="F5" s="26" t="n"/>
+          <t>PHẦN KHÓ NHẤT: Vòng đời Booking &amp; State Machine, Concurrency Locking chống trùng xe, Schedulers tự động hóa, Giao - Trả xe &amp; Phụ phí (US-06, US-07, US-09, US-10)</t>
+        </is>
+      </c>
+      <c r="F5" s="26" t="inlineStr">
+        <is>
+          <t>Backend Chủ lực (Core logic)</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="24.75" customHeight="1">
       <c r="A6" s="28" t="n">
@@ -3845,21 +3842,25 @@
       </c>
       <c r="B6" s="26" t="inlineStr">
         <is>
-          <t>Khiêm</t>
-        </is>
-      </c>
-      <c r="C6" s="28" t="n"/>
+          <t>Chí Vĩ</t>
+        </is>
+      </c>
+      <c r="C6" s="28" t="inlineStr"/>
       <c r="D6" s="25" t="inlineStr">
         <is>
-          <t>Backend Developer</t>
+          <t>Backend Developer (Auth &amp; Admin)</t>
         </is>
       </c>
       <c r="E6" s="26" t="inlineStr">
         <is>
-          <t>Sprint 0 (Luồng 2), BE Trans: US-02, US-07, US-08, US-09, US-10, US-11, US-12, US-13, US-15</t>
-        </is>
-      </c>
-      <c r="F6" s="26" t="n"/>
+          <t>Xác thực &amp; Phân quyền RBAC, Quản lý User/Profile, Trang Quản trị Admin &amp; Dashboard (US-01, US-02, US-14)</t>
+        </is>
+      </c>
+      <c r="F6" s="26" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="24.75" customHeight="1">
       <c r="A7" s="28" t="n">
@@ -3867,21 +3868,25 @@
       </c>
       <c r="B7" s="26" t="inlineStr">
         <is>
-          <t>Quân</t>
-        </is>
-      </c>
-      <c r="C7" s="28" t="n"/>
+          <t>Phát</t>
+        </is>
+      </c>
+      <c r="C7" s="28" t="inlineStr"/>
       <c r="D7" s="25" t="inlineStr">
         <is>
-          <t>Frontend Developer</t>
+          <t>Backend Developer (Car &amp; Search &amp; AI)</t>
         </is>
       </c>
       <c r="E7" s="26" t="inlineStr">
         <is>
-          <t>Sprint 0 (DB Catalog), FE Core: US-01, US-02, US-03, US-05, US-06, US-08, US-09, US-10, US-11</t>
-        </is>
-      </c>
-      <c r="F7" s="26" t="n"/>
+          <t>Quản lý xe cho thuê, Bộ lọc tìm kiếm động, Tích hợp AI gợi ý &amp; tóm tắt (US-03, US-04, US-05, US-15)</t>
+        </is>
+      </c>
+      <c r="F7" s="26" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="24.75" customHeight="1">
       <c r="A8" s="28" t="n">
@@ -3889,21 +3894,51 @@
       </c>
       <c r="B8" s="26" t="inlineStr">
         <is>
-          <t>Tín</t>
-        </is>
-      </c>
-      <c r="C8" s="28" t="n"/>
+          <t>Quân</t>
+        </is>
+      </c>
+      <c r="C8" s="28" t="inlineStr"/>
       <c r="D8" s="25" t="inlineStr">
         <is>
-          <t>Tester / QA</t>
+          <t>Backend Developer (Payment &amp; Services)</t>
         </is>
       </c>
       <c r="E8" s="26" t="inlineStr">
         <is>
-          <t>Sprint 0 (QA Gatekeeper), Test &amp; QA toàn bộ 15 Stories (Subtasks Test)</t>
-        </is>
-      </c>
-      <c r="F8" s="26" t="n"/>
+          <t>Hỗ trợ BE Thanh toán &amp; Lịch sử giao dịch, Đánh giá, Khiếu nại, WebSocket Thông báo (US-08, US-11, US-12, US-13)</t>
+        </is>
+      </c>
+      <c r="F8" s="26" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="26" t="inlineStr">
+        <is>
+          <t>Chí Tín</t>
+        </is>
+      </c>
+      <c r="C9" s="28" t="inlineStr"/>
+      <c r="D9" s="25" t="inlineStr">
+        <is>
+          <t>Frontend / QA &amp; Tester (Chuyên gia Thanh toán)</t>
+        </is>
+      </c>
+      <c r="E9" s="26" t="inlineStr">
+        <is>
+          <t>Xây dựng UI Web Frontend, Phụ trách luồng Thanh toán (kinh nghiệm Payment), QA Gatekeeper &amp; Kiểm thử toàn bộ 15 Stories</t>
+        </is>
+      </c>
+      <c r="F9" s="26" t="inlineStr">
+        <is>
+          <t>FE + Test + Payment Specialist</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>